<commit_message>
Refine demo weekly sample calculations
Adds current-week fictional records, prevents awards for zero production, and auto-loads the sample workbook for demo logins.
</commit_message>
<xml_diff>
--- a/A사_가상실적_시상데모.xlsx
+++ b/A사_가상실적_시상데모.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" r:id="R12fa7818af804ffd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실적데이터" sheetId="2" r:id="R8d711f405cd04fd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시상규칙" sheetId="3" r:id="Rb9d4a3cea22d4201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" r:id="Re65f48d03c054216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실적데이터" sheetId="2" r:id="R0265def9ab4e4fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시상규칙" sheetId="3" r:id="R147fd132769c443e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -779,6 +779,181 @@
         <x:v>가상자료</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>DEMO-A</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>가상 부산지사</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>30000001</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>70000001</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>가상설계사A</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>가상건강플랜</x:v>
+      </x:c>
+      <x:c r="H14" t="n">
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="I14" t="n">
+        <x:v>600000</x:v>
+      </x:c>
+      <x:c r="J14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>가상자료</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>DEMO-A</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>가상 부산지사</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>30000001</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>70000002</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>가상설계사B</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>가상건강플랜</x:v>
+      </x:c>
+      <x:c r="H15" t="n">
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="I15" t="n">
+        <x:v>600000</x:v>
+      </x:c>
+      <x:c r="J15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>가상자료</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>DEMO-A</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>가상 부산지사</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>30000001</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>70000003</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>가상설계사C</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>가상건강플랜</x:v>
+      </x:c>
+      <x:c r="H16" t="n">
+        <x:v>40000</x:v>
+      </x:c>
+      <x:c r="I16" t="n">
+        <x:v>400000</x:v>
+      </x:c>
+      <x:c r="J16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>가상자료</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>DEMO-A</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>가상 부산지사</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>30000001</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>70000004</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>가상설계사D</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>가상든든플랜</x:v>
+      </x:c>
+      <x:c r="H17" t="n">
+        <x:v>65000</x:v>
+      </x:c>
+      <x:c r="I17" t="n">
+        <x:v>650000</x:v>
+      </x:c>
+      <x:c r="J17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>가상자료</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>DEMO-A</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>가상 부산지사</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>30000001</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>70000005</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>가상설계사E</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>가상건강플랜</x:v>
+      </x:c>
+      <x:c r="H18" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="I18" t="n">
+        <x:v>200000</x:v>
+      </x:c>
+      <x:c r="J18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>가상자료</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Publish A-D demo and manager scope
Synthetic four-company demo data, award guides, and cross-company manager visibility.
</commit_message>
<xml_diff>
--- a/A사_가상실적_시상데모.xlsx
+++ b/A사_가상실적_시상데모.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" r:id="Re65f48d03c054216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실적데이터" sheetId="2" r:id="R0265def9ab4e4fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시상규칙" sheetId="3" r:id="R147fd132769c443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" r:id="R1853e6e6e0934e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실적데이터" sheetId="2" r:id="R190349f399f44a8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시상규칙" sheetId="3" r:id="R0a9b1b0742ca465b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +36,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF187B63"/>
+        <x:fgColor rgb="FF8B1015"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -260,10 +260,10 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>A사 실적·시상 데모</x:v>
+        <x:v>A사 가상 데모</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str">
-        <x:v>가상자료 안내</x:v>
+        <x:v>자료 안내</x:v>
       </x:c>
       <x:c r="C1" s="2"/>
       <x:c r="D1" s="2"/>
@@ -280,7 +280,7 @@
         <x:v>자료 성격</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>교육·화면 시연용 가상 데이터</x:v>
+        <x:v>완전 가상 · 화면 점검용</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -288,31 +288,63 @@
         <x:v>기준 월</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>2026년 10월 (예시)</x:v>
+        <x:v>2026년 10월 (가상 예시)</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>시상 방식</x:v>
+        <x:v>대리점 코드</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>해당 구간 도달 시 해당 구간 시상금만 지급 (누적 아님)</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>로그인 예시</x:v>
+        <x:v>예시 매니저 코드</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>설계사 70000001 / 매니저 30000001</x:v>
+        <x:v>30000001</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>주의</x:v>
+        <x:v>예시 설계사 코드</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>실제 회사·대리점·실적·시상 규칙과 무관합니다.</x:v>
+        <x:v>70000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>주차 시상 방식</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>월납P 구간 도달 시 그 구간 지급액만 지급 (누적 아님)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>지급 조건</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>13회차 유지 확인 후 익월 지급</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>월납P 배수 예시</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>당월 260% · 2차년도 170% (기준 월납P 10만원 가정)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>중요</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>실제 회사·대리점의 기준이나 지급 약속이 아닙니다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -361,10 +393,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>30000001</x:v>
@@ -373,19 +405,19 @@
         <x:v>70000001</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>가상설계사A</x:v>
+        <x:v>가상A설계사1</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>2026-10-02</x:v>
+        <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상인보험</x:v>
       </x:c>
       <x:c r="H2" t="n">
-        <x:v>40000</x:v>
+        <x:v>70000</x:v>
       </x:c>
       <x:c r="I2" t="n">
-        <x:v>400000</x:v>
+        <x:v>700000</x:v>
       </x:c>
       <x:c r="J2" t="n">
         <x:v>1</x:v>
@@ -396,10 +428,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C3" t="str">
         <x:v>30000001</x:v>
@@ -408,19 +440,19 @@
         <x:v>70000001</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>가상설계사A</x:v>
+        <x:v>가상A설계사1</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>2026-10-06</x:v>
+        <x:v>2026-10-10</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상통합건강</x:v>
       </x:c>
       <x:c r="H3" t="n">
-        <x:v>35000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="I3" t="n">
-        <x:v>350000</x:v>
+        <x:v>800000</x:v>
       </x:c>
       <x:c r="J3" t="n">
         <x:v>1</x:v>
@@ -431,10 +463,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C4" t="str">
         <x:v>30000001</x:v>
@@ -443,19 +475,19 @@
         <x:v>70000001</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>가상설계사A</x:v>
+        <x:v>가상A설계사1</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>2026-10-10</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>가상든든플랜</x:v>
+        <x:v>가상간편</x:v>
       </x:c>
       <x:c r="H4" t="n">
-        <x:v>45000</x:v>
+        <x:v>110000</x:v>
       </x:c>
       <x:c r="I4" t="n">
-        <x:v>450000</x:v>
+        <x:v>1100000</x:v>
       </x:c>
       <x:c r="J4" t="n">
         <x:v>1</x:v>
@@ -466,31 +498,31 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>30000001</x:v>
+        <x:v>30000004</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>70000001</x:v>
+        <x:v>70000002</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>가상설계사A</x:v>
+        <x:v>가상A설계사2</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>2026-10-14</x:v>
+        <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상인보험</x:v>
       </x:c>
       <x:c r="H5" t="n">
-        <x:v>30000</x:v>
+        <x:v>140000</x:v>
       </x:c>
       <x:c r="I5" t="n">
-        <x:v>300000</x:v>
+        <x:v>1400000</x:v>
       </x:c>
       <x:c r="J5" t="n">
         <x:v>1</x:v>
@@ -501,34 +533,34 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>30000001</x:v>
+        <x:v>30000004</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>70000002</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>가상설계사B</x:v>
+        <x:v>가상A설계사2</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-10</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상통합건강</x:v>
       </x:c>
       <x:c r="H6" t="n">
-        <x:v>90000</x:v>
+        <x:v>190000</x:v>
       </x:c>
       <x:c r="I6" t="n">
-        <x:v>900000</x:v>
+        <x:v>1900000</x:v>
       </x:c>
       <x:c r="J6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K6" t="str">
         <x:v>가상자료</x:v>
@@ -536,31 +568,31 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>30000001</x:v>
+        <x:v>30000004</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>70000002</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>가상설계사B</x:v>
+        <x:v>가상A설계사2</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>2026-10-11</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>가상든든플랜</x:v>
+        <x:v>가상간편</x:v>
       </x:c>
       <x:c r="H7" t="n">
-        <x:v>10000</x:v>
+        <x:v>80000</x:v>
       </x:c>
       <x:c r="I7" t="n">
-        <x:v>100000</x:v>
+        <x:v>800000</x:v>
       </x:c>
       <x:c r="J7" t="n">
         <x:v>1</x:v>
@@ -571,10 +603,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>30000001</x:v>
@@ -583,19 +615,19 @@
         <x:v>70000003</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>가상설계사C</x:v>
+        <x:v>가상A설계사3</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상인보험</x:v>
       </x:c>
       <x:c r="H8" t="n">
-        <x:v>50000</x:v>
+        <x:v>280000</x:v>
       </x:c>
       <x:c r="I8" t="n">
-        <x:v>500000</x:v>
+        <x:v>2800000</x:v>
       </x:c>
       <x:c r="J8" t="n">
         <x:v>1</x:v>
@@ -606,10 +638,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>30000001</x:v>
@@ -618,22 +650,22 @@
         <x:v>70000003</x:v>
       </x:c>
       <x:c r="E9" t="str">
-        <x:v>가상설계사C</x:v>
+        <x:v>가상A설계사3</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>2026-10-13</x:v>
+        <x:v>2026-10-10</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>가상든든플랜</x:v>
+        <x:v>가상통합건강</x:v>
       </x:c>
       <x:c r="H9" t="n">
-        <x:v>65000</x:v>
+        <x:v>220000</x:v>
       </x:c>
       <x:c r="I9" t="n">
-        <x:v>650000</x:v>
+        <x:v>2200000</x:v>
       </x:c>
       <x:c r="J9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K9" t="str">
         <x:v>가상자료</x:v>
@@ -641,316 +673,36 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>가상 부산지사</x:v>
+        <x:v>가상 A사 지사</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>30000001</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>70000004</x:v>
+        <x:v>70000003</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>가상설계사D</x:v>
+        <x:v>가상A설계사3</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>2026-10-08</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상간편</x:v>
       </x:c>
       <x:c r="H10" t="n">
-        <x:v>20000</x:v>
+        <x:v>150000</x:v>
       </x:c>
       <x:c r="I10" t="n">
-        <x:v>200000</x:v>
+        <x:v>1500000</x:v>
       </x:c>
       <x:c r="J10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D11" t="str">
-        <x:v>70000004</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>가상설계사D</x:v>
-      </x:c>
-      <x:c r="F11" t="str">
-        <x:v>2026-10-15</x:v>
-      </x:c>
-      <x:c r="G11" t="str">
-        <x:v>가상든든플랜</x:v>
-      </x:c>
-      <x:c r="H11" t="n">
-        <x:v>25000</x:v>
-      </x:c>
-      <x:c r="I11" t="n">
-        <x:v>250000</x:v>
-      </x:c>
-      <x:c r="J11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K11" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D12" t="str">
-        <x:v>70000005</x:v>
-      </x:c>
-      <x:c r="E12" t="str">
-        <x:v>가상설계사E</x:v>
-      </x:c>
-      <x:c r="F12" t="str">
-        <x:v>2026-10-03</x:v>
-      </x:c>
-      <x:c r="G12" t="str">
-        <x:v>가상건강플랜</x:v>
-      </x:c>
-      <x:c r="H12" t="n">
-        <x:v>120000</x:v>
-      </x:c>
-      <x:c r="I12" t="n">
-        <x:v>1200000</x:v>
-      </x:c>
-      <x:c r="J12" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="K12" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D13" t="str">
-        <x:v>70000005</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
-        <x:v>가상설계사E</x:v>
-      </x:c>
-      <x:c r="F13" t="str">
-        <x:v>2026-10-12</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
-        <x:v>가상든든플랜</x:v>
-      </x:c>
-      <x:c r="H13" t="n">
-        <x:v>40000</x:v>
-      </x:c>
-      <x:c r="I13" t="n">
-        <x:v>400000</x:v>
-      </x:c>
-      <x:c r="J13" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K13" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>70000001</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>가상설계사A</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>2026-10-15</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>가상건강플랜</x:v>
-      </x:c>
-      <x:c r="H14" t="n">
-        <x:v>60000</x:v>
-      </x:c>
-      <x:c r="I14" t="n">
-        <x:v>600000</x:v>
-      </x:c>
-      <x:c r="J14" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K14" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>70000002</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>가상설계사B</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>2026-10-15</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>가상건강플랜</x:v>
-      </x:c>
-      <x:c r="H15" t="n">
-        <x:v>60000</x:v>
-      </x:c>
-      <x:c r="I15" t="n">
-        <x:v>600000</x:v>
-      </x:c>
-      <x:c r="J15" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K15" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>70000003</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>가상설계사C</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>2026-10-15</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>가상건강플랜</x:v>
-      </x:c>
-      <x:c r="H16" t="n">
-        <x:v>40000</x:v>
-      </x:c>
-      <x:c r="I16" t="n">
-        <x:v>400000</x:v>
-      </x:c>
-      <x:c r="J16" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K16" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>70000004</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>가상설계사D</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>2026-10-15</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
-        <x:v>가상든든플랜</x:v>
-      </x:c>
-      <x:c r="H17" t="n">
-        <x:v>65000</x:v>
-      </x:c>
-      <x:c r="I17" t="n">
-        <x:v>650000</x:v>
-      </x:c>
-      <x:c r="J17" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K17" t="str">
-        <x:v>가상자료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>DEMO-A</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>가상 부산지사</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>30000001</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>70000005</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>가상설계사E</x:v>
-      </x:c>
-      <x:c r="F18" t="str">
-        <x:v>2026-10-15</x:v>
-      </x:c>
-      <x:c r="G18" t="str">
-        <x:v>가상건강플랜</x:v>
-      </x:c>
-      <x:c r="H18" t="n">
-        <x:v>20000</x:v>
-      </x:c>
-      <x:c r="I18" t="n">
-        <x:v>200000</x:v>
-      </x:c>
-      <x:c r="J18" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K18" t="str">
         <x:v>가상자료</x:v>
       </x:c>
     </x:row>
@@ -986,7 +738,7 @@
         <x:v>시상금(원)</x:v>
       </x:c>
       <x:c r="H1" s="2" t="str">
-        <x:v>지급/유지 조건</x:v>
+        <x:v>지급·유지 조건</x:v>
       </x:c>
       <x:c r="I1" s="2"/>
       <x:c r="J1" s="2"/>
@@ -997,25 +749,25 @@
         <x:v>주차</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>2026-10-01~2026-10-31</x:v>
+        <x:v>2026-10</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>전체 월납P</x:v>
       </x:c>
       <x:c r="E2" t="n">
-        <x:v>0</x:v>
+        <x:v>100000</x:v>
       </x:c>
       <x:c r="F2" t="n">
-        <x:v>49999</x:v>
+        <x:v>199999</x:v>
       </x:c>
       <x:c r="G2" t="n">
-        <x:v>5000</x:v>
+        <x:v>100000</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>구간별 단일 지급 · 가상</x:v>
+        <x:v>13회차 유지 확인 후 익월 지급 · 해당 구간만 지급</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1023,25 +775,25 @@
         <x:v>주차</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>2026-10-01~2026-10-31</x:v>
+        <x:v>2026-10</x:v>
       </x:c>
       <x:c r="D3" t="str">
         <x:v>전체 월납P</x:v>
       </x:c>
       <x:c r="E3" t="n">
-        <x:v>50000</x:v>
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="F3" t="n">
-        <x:v>99999</x:v>
+        <x:v>299999</x:v>
       </x:c>
       <x:c r="G3" t="n">
-        <x:v>10000</x:v>
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>구간별 단일 지급 · 가상</x:v>
+        <x:v>13회차 유지 확인 후 익월 지급 · 해당 구간만 지급</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1049,25 +801,25 @@
         <x:v>주차</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>2026-10-01~2026-10-31</x:v>
+        <x:v>2026-10</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>전체 월납P</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>100000</x:v>
+        <x:v>300000</x:v>
       </x:c>
       <x:c r="F4" t="n">
-        <x:v>199999</x:v>
+        <x:v>499999</x:v>
       </x:c>
       <x:c r="G4" t="n">
-        <x:v>20000</x:v>
+        <x:v>300000</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>구간별 단일 지급 · 가상</x:v>
+        <x:v>13회차 유지 확인 후 익월 지급 · 해당 구간만 지급</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1075,25 +827,25 @@
         <x:v>주차</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>2026-10-01~2026-10-31</x:v>
+        <x:v>2026-10</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>전체 월납P</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>200000</x:v>
+        <x:v>500000</x:v>
       </x:c>
       <x:c r="F5" t="n">
         <x:v>999999999</x:v>
       </x:c>
       <x:c r="G5" t="n">
-        <x:v>40000</x:v>
+        <x:v>500000</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>구간별 단일 지급 · 가상</x:v>
+        <x:v>13회차 유지 확인 후 익월 지급 · 해당 구간만 지급</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1101,39 +853,39 @@
         <x:v>상품추가</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>2026-10-01~2026-10-31</x:v>
+        <x:v>2026-10</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>가상건강플랜</x:v>
+        <x:v>가상통합건강</x:v>
       </x:c>
       <x:c r="E6" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="F6" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G6" t="n">
         <x:v>30000</x:v>
       </x:c>
-      <x:c r="F6" t="n">
-        <x:v>999999999</x:v>
-      </x:c>
-      <x:c r="G6" t="n">
-        <x:v>3000</x:v>
-      </x:c>
       <x:c r="H6" t="str">
-        <x:v>상품 대상·추가 시상은 데모 예시</x:v>
+        <x:v>대상 상품 월납P 기준 · 가상</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>연속가동</x:v>
+        <x:v>상품추가</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>DEMO-A</x:v>
+        <x:v>AG-A</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>가상기간</x:v>
+        <x:v>2026-10</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>가상든든플랜</x:v>
+        <x:v>가상간편</x:v>
       </x:c>
       <x:c r="E7" t="n">
         <x:v>100000</x:v>
@@ -1142,10 +894,384 @@
         <x:v>999999999</x:v>
       </x:c>
       <x:c r="G7" t="n">
-        <x:v>15000</x:v>
+        <x:v>30000</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>가상 익월 조건 · 누적 아님</x:v>
+        <x:v>대상 상품 월납P 기준 · 가상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>상품추가</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>2026-10</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>가상어린이</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="F8" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G8" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>대상 상품 월납P 기준 · 가상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>정규 월납P 비율</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>가상 월간</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>인보험</x:v>
+      </x:c>
+      <x:c r="E9"/>
+      <x:c r="F9"/>
+      <x:c r="G9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>월납P × 100% · 13회차 유지 확인 후 익월 지급</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>정규 월납P 비율</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>가상 월간</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>재물·단체</x:v>
+      </x:c>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>월납P × 100% · 13회차 유지 확인 후 익월 지급</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>정규 월납P 비율</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>가상 월간</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>펫퍼민트</x:v>
+      </x:c>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>월납P × 300% · 13회차 유지 확인 후 익월 지급</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>월납P 배수</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>가상 월간</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>익월 지급 시상</x:v>
+      </x:c>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12" t="n">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>월납P × 260% · 기준 월납P 10만원 예시 · 13회차 유지 확인 후 익월 지급</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>2차년도</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>가상 월간</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>2차년도 유지</x:v>
+      </x:c>
+      <x:c r="E13" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="F13" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G13" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>월납P × 170% · 13회차 등 유지 기준은 회사별 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>연속가동</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>2026-10-15~2026-11-19</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>직전기간 월납P 10만원 구간</x:v>
+      </x:c>
+      <x:c r="E14" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="F14" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G14" t="n">
+        <x:v>200000</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>다음달 1~19일 월납P 10만원 달성 시 지급 · 구간별 단일 지급 · 누적 아님</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>연속가동</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>2026-10-15~2026-11-19</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>직전기간 월납P 20만원 구간</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>200000</x:v>
+      </x:c>
+      <x:c r="F15" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G15" t="n">
+        <x:v>600000</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>다음달 1~19일 월납P 10만원 달성 시 지급 · 구간별 단일 지급 · 누적 아님</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>연속가동</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>2026-10-15~2026-11-19</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>직전기간 월납P 30만원 구간</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="F16" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G16" t="n">
+        <x:v>800000</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>다음달 1~19일 월납P 10만원 달성 시 지급 · 구간별 단일 지급 · 누적 아님</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>연속가동</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>2026-10-15~2026-11-19</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>직전기간 월납P 50만원 구간</x:v>
+      </x:c>
+      <x:c r="E17" t="n">
+        <x:v>500000</x:v>
+      </x:c>
+      <x:c r="F17" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G17" t="n">
+        <x:v>1800000</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>다음달 1~19일 월납P 10만원 달성 시 지급 · 구간별 단일 지급 · 누적 아님</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>MC PLUS</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>가상 연속 기간</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>월납P 20만원 구간</x:v>
+      </x:c>
+      <x:c r="E18" t="n">
+        <x:v>200000</x:v>
+      </x:c>
+      <x:c r="F18" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G18" t="n">
+        <x:v>600000</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>해당 구간 지급 예시 · 누적 방식은 가상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>MC PLUS</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>가상 연속 기간</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>월납P 40만원 구간</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
+        <x:v>400000</x:v>
+      </x:c>
+      <x:c r="F19" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G19" t="n">
+        <x:v>1200000</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>해당 구간 지급 예시 · 누적 방식은 가상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>MC PLUS</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>가상 연속 기간</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>월납P 60만원 구간</x:v>
+      </x:c>
+      <x:c r="E20" t="n">
+        <x:v>600000</x:v>
+      </x:c>
+      <x:c r="F20" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G20" t="n">
+        <x:v>1800000</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>해당 구간 지급 예시 · 누적 방식은 가상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>MC PLUS</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>가상 연속 기간</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>월납P 80만원 구간</x:v>
+      </x:c>
+      <x:c r="E21" t="n">
+        <x:v>800000</x:v>
+      </x:c>
+      <x:c r="F21" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G21" t="n">
+        <x:v>2400000</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>해당 구간 지급 예시 · 누적 방식은 가상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>MC PLUS</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>AG-A</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>가상 연속 기간</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>월납P 100만원 구간</x:v>
+      </x:c>
+      <x:c r="E22" t="n">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="F22" t="n">
+        <x:v>999999999</x:v>
+      </x:c>
+      <x:c r="G22" t="n">
+        <x:v>3000000</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>해당 구간 지급 예시 · 누적 방식은 가상</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>